<commit_message>
fix: use external templates for attendance export
</commit_message>
<xml_diff>
--- a/templates/attendance(2025)_template.xlsx
+++ b/templates/attendance(2025)_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ss962\Documents\attendance\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ss962\Documents\attendance\dist\win-unpacked\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C976D0E-78FB-4C99-B1BB-841D1FC6F573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28127B8A-9C1B-403F-AE27-E77192A95480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -991,15 +991,7 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>김민성</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>윤찬희</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>정찬민</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
@@ -1008,6 +1000,14 @@
   </si>
   <si>
     <t>C-arm</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>고영수</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>이이정</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1917,29 +1917,20 @@
     <xf numFmtId="180" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="5" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1965,20 +1956,29 @@
     <xf numFmtId="0" fontId="17" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="41" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="5" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="6" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -1991,22 +1991,7 @@
     <cellStyle name="표준 2 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="표준 4" xfId="6" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF002060"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -2019,22 +2004,12 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FFFF0000"/>
+        <color rgb="FFC00000"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
+        <color rgb="FF002060"/>
       </font>
     </dxf>
     <dxf>
@@ -3865,30 +3840,30 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="AJ6:AJ7">
-    <cfRule type="cellIs" dxfId="14" priority="5" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="6" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="8" priority="6" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ9">
-    <cfRule type="cellIs" dxfId="12" priority="4" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="7" priority="4" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ9:AJ10">
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ12 AJ15 AJ18 AJ21 AJ24 AJ27">
-    <cfRule type="cellIs" dxfId="10" priority="2" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="5" priority="2" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ12:AJ13 AJ15:AJ16 AJ18:AJ19 AJ21:AJ22 AJ24:AJ25 AJ27:AJ28">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4146,7 +4121,7 @@
         <v>80</v>
       </c>
       <c r="AM4" s="86" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:39" ht="20.25" customHeight="1">
@@ -4201,7 +4176,7 @@
         <v>81</v>
       </c>
       <c r="AM5" s="86" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:39" ht="20.25" customHeight="1">
@@ -4247,10 +4222,10 @@
         <v>0</v>
       </c>
       <c r="AL6" s="86" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AM6" s="86" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:39" ht="20.25" customHeight="1">
@@ -4300,10 +4275,10 @@
         <v>0</v>
       </c>
       <c r="AL7" s="86" t="s">
+        <v>85</v>
+      </c>
+      <c r="AM7" s="86" t="s">
         <v>83</v>
-      </c>
-      <c r="AM7" s="86" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:39" ht="20.25" customHeight="1">
@@ -4487,19 +4462,19 @@
     <row r="36" ht="20.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="AJ6:AJ7">
-    <cfRule type="cellIs" dxfId="6" priority="11" operator="greaterThanOrEqual">
+  <conditionalFormatting sqref="AJ5:AJ1048576">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="12" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ5:AJ1048576">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="AJ6:AJ7">
+    <cfRule type="cellIs" dxfId="1" priority="11" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="12" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4536,32 +4511,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" s="16" customFormat="1" ht="21" customHeight="1">
-      <c r="A1" s="145"/>
-      <c r="B1" s="145"/>
-      <c r="C1" s="145"/>
+      <c r="A1" s="142"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
       <c r="D1" s="50"/>
-      <c r="E1" s="146" t="s">
+      <c r="E1" s="143" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="146"/>
-      <c r="G1" s="147" t="s">
+      <c r="F1" s="143"/>
+      <c r="G1" s="144" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="147"/>
-      <c r="I1" s="147"/>
-      <c r="J1" s="147"/>
-      <c r="K1" s="149">
+      <c r="H1" s="144"/>
+      <c r="I1" s="144"/>
+      <c r="J1" s="144"/>
+      <c r="K1" s="146">
         <v>9</v>
       </c>
-      <c r="L1" s="151" t="s">
+      <c r="L1" s="148" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="151"/>
-      <c r="N1" s="151"/>
-      <c r="O1" s="151"/>
-      <c r="P1" s="151"/>
-      <c r="Q1" s="151"/>
-      <c r="R1" s="151"/>
+      <c r="M1" s="148"/>
+      <c r="N1" s="148"/>
+      <c r="O1" s="148"/>
+      <c r="P1" s="148"/>
+      <c r="Q1" s="148"/>
+      <c r="R1" s="148"/>
       <c r="S1" s="57"/>
       <c r="T1" s="58"/>
       <c r="U1" s="58" t="s">
@@ -4583,24 +4558,24 @@
       <c r="AH1" s="17"/>
     </row>
     <row r="2" spans="1:35" s="16" customFormat="1" ht="21" customHeight="1" thickBot="1">
-      <c r="A2" s="145"/>
-      <c r="B2" s="145"/>
-      <c r="C2" s="145"/>
+      <c r="A2" s="142"/>
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
       <c r="D2" s="50"/>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="148"/>
-      <c r="H2" s="148"/>
-      <c r="I2" s="148"/>
-      <c r="J2" s="148"/>
-      <c r="K2" s="150"/>
-      <c r="L2" s="152"/>
-      <c r="M2" s="152"/>
-      <c r="N2" s="152"/>
-      <c r="O2" s="152"/>
-      <c r="P2" s="152"/>
-      <c r="Q2" s="152"/>
-      <c r="R2" s="152"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="145"/>
+      <c r="H2" s="145"/>
+      <c r="I2" s="145"/>
+      <c r="J2" s="145"/>
+      <c r="K2" s="147"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
+      <c r="O2" s="149"/>
+      <c r="P2" s="149"/>
+      <c r="Q2" s="149"/>
+      <c r="R2" s="149"/>
       <c r="S2" s="59"/>
       <c r="T2" s="58"/>
       <c r="U2" s="58" t="s">
@@ -4658,41 +4633,41 @@
       <c r="AH3" s="17"/>
     </row>
     <row r="4" spans="1:35" s="14" customFormat="1" ht="15" customHeight="1">
-      <c r="A4" s="144" t="str">
+      <c r="A4" s="156" t="str">
         <f>A1&amp;" "&amp;C1</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="B4" s="144"/>
-      <c r="C4" s="144"/>
-      <c r="D4" s="144"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
       <c r="E4" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="144" t="s">
+      <c r="F4" s="156" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="144"/>
-      <c r="H4" s="144"/>
-      <c r="I4" s="144"/>
-      <c r="J4" s="144"/>
-      <c r="K4" s="144"/>
-      <c r="L4" s="144"/>
-      <c r="M4" s="144" t="s">
+      <c r="G4" s="156"/>
+      <c r="H4" s="156"/>
+      <c r="I4" s="156"/>
+      <c r="J4" s="156"/>
+      <c r="K4" s="156"/>
+      <c r="L4" s="156"/>
+      <c r="M4" s="156" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="144"/>
-      <c r="O4" s="144"/>
-      <c r="P4" s="144"/>
-      <c r="Q4" s="144"/>
-      <c r="R4" s="144"/>
-      <c r="S4" s="144"/>
-      <c r="T4" s="140" t="s">
+      <c r="N4" s="156"/>
+      <c r="O4" s="156"/>
+      <c r="P4" s="156"/>
+      <c r="Q4" s="156"/>
+      <c r="R4" s="156"/>
+      <c r="S4" s="156"/>
+      <c r="T4" s="150" t="s">
         <v>15</v>
       </c>
-      <c r="U4" s="140" t="s">
+      <c r="U4" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="V4" s="140" t="s">
+      <c r="V4" s="150" t="s">
         <v>17</v>
       </c>
       <c r="W4" s="15"/>
@@ -4710,30 +4685,30 @@
       <c r="AI4" s="15"/>
     </row>
     <row r="5" spans="1:35" s="14" customFormat="1" ht="15" customHeight="1">
-      <c r="A5" s="144"/>
-      <c r="B5" s="144"/>
-      <c r="C5" s="144"/>
-      <c r="D5" s="144"/>
-      <c r="E5" s="141" t="s">
+      <c r="A5" s="156"/>
+      <c r="B5" s="156"/>
+      <c r="C5" s="156"/>
+      <c r="D5" s="156"/>
+      <c r="E5" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="144"/>
-      <c r="G5" s="144"/>
-      <c r="H5" s="144"/>
-      <c r="I5" s="144"/>
-      <c r="J5" s="144"/>
-      <c r="K5" s="144"/>
-      <c r="L5" s="144"/>
-      <c r="M5" s="144"/>
-      <c r="N5" s="144"/>
-      <c r="O5" s="144"/>
-      <c r="P5" s="144"/>
-      <c r="Q5" s="144"/>
-      <c r="R5" s="144"/>
-      <c r="S5" s="144"/>
-      <c r="T5" s="140"/>
-      <c r="U5" s="140"/>
-      <c r="V5" s="140"/>
+      <c r="F5" s="156"/>
+      <c r="G5" s="156"/>
+      <c r="H5" s="156"/>
+      <c r="I5" s="156"/>
+      <c r="J5" s="156"/>
+      <c r="K5" s="156"/>
+      <c r="L5" s="156"/>
+      <c r="M5" s="156"/>
+      <c r="N5" s="156"/>
+      <c r="O5" s="156"/>
+      <c r="P5" s="156"/>
+      <c r="Q5" s="156"/>
+      <c r="R5" s="156"/>
+      <c r="S5" s="156"/>
+      <c r="T5" s="150"/>
+      <c r="U5" s="150"/>
+      <c r="V5" s="150"/>
       <c r="W5" s="15"/>
       <c r="X5" s="15"/>
       <c r="Y5" s="15"/>
@@ -4749,60 +4724,60 @@
       <c r="AI5" s="15"/>
     </row>
     <row r="6" spans="1:35" s="14" customFormat="1" ht="15" customHeight="1">
-      <c r="A6" s="142" t="s">
+      <c r="A6" s="152" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="143" t="s">
+      <c r="B6" s="153" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="143" t="s">
+      <c r="C6" s="153" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="138" t="s">
+      <c r="D6" s="154" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="141"/>
-      <c r="F6" s="139" t="s">
+      <c r="E6" s="151"/>
+      <c r="F6" s="155" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="139" t="s">
+      <c r="G6" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="138" t="s">
+      <c r="H6" s="154" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="138"/>
-      <c r="J6" s="137" t="s">
+      <c r="I6" s="154"/>
+      <c r="J6" s="157" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="138" t="s">
+      <c r="K6" s="154" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="137" t="s">
+      <c r="L6" s="157" t="s">
         <v>6</v>
       </c>
-      <c r="M6" s="139" t="s">
+      <c r="M6" s="155" t="s">
         <v>22</v>
       </c>
-      <c r="N6" s="139" t="s">
+      <c r="N6" s="155" t="s">
         <v>23</v>
       </c>
-      <c r="O6" s="138" t="s">
+      <c r="O6" s="154" t="s">
         <v>24</v>
       </c>
-      <c r="P6" s="138"/>
-      <c r="Q6" s="137" t="s">
+      <c r="P6" s="154"/>
+      <c r="Q6" s="157" t="s">
         <v>27</v>
       </c>
-      <c r="R6" s="138" t="s">
+      <c r="R6" s="154" t="s">
         <v>26</v>
       </c>
-      <c r="S6" s="137" t="s">
+      <c r="S6" s="157" t="s">
         <v>28</v>
       </c>
-      <c r="T6" s="140"/>
-      <c r="U6" s="140"/>
-      <c r="V6" s="140"/>
+      <c r="T6" s="150"/>
+      <c r="U6" s="150"/>
+      <c r="V6" s="150"/>
       <c r="W6" s="15"/>
       <c r="X6" s="15"/>
       <c r="Y6" s="15"/>
@@ -4818,36 +4793,36 @@
       <c r="AI6" s="15"/>
     </row>
     <row r="7" spans="1:35" s="14" customFormat="1" ht="24" customHeight="1">
-      <c r="A7" s="142"/>
-      <c r="B7" s="143"/>
-      <c r="C7" s="143"/>
-      <c r="D7" s="138"/>
-      <c r="E7" s="141"/>
-      <c r="F7" s="139"/>
-      <c r="G7" s="139"/>
+      <c r="A7" s="152"/>
+      <c r="B7" s="153"/>
+      <c r="C7" s="153"/>
+      <c r="D7" s="154"/>
+      <c r="E7" s="151"/>
+      <c r="F7" s="155"/>
+      <c r="G7" s="155"/>
       <c r="H7" s="74" t="s">
         <v>29</v>
       </c>
       <c r="I7" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="137"/>
-      <c r="K7" s="138"/>
-      <c r="L7" s="137"/>
-      <c r="M7" s="139"/>
-      <c r="N7" s="139"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="154"/>
+      <c r="L7" s="157"/>
+      <c r="M7" s="155"/>
+      <c r="N7" s="155"/>
       <c r="O7" s="75" t="s">
         <v>29</v>
       </c>
       <c r="P7" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="Q7" s="137"/>
-      <c r="R7" s="138"/>
-      <c r="S7" s="137"/>
-      <c r="T7" s="140"/>
-      <c r="U7" s="140"/>
-      <c r="V7" s="140"/>
+      <c r="Q7" s="157"/>
+      <c r="R7" s="154"/>
+      <c r="S7" s="157"/>
+      <c r="T7" s="150"/>
+      <c r="U7" s="150"/>
+      <c r="V7" s="150"/>
       <c r="W7" s="15"/>
       <c r="X7" s="15"/>
       <c r="Y7" s="15"/>
@@ -5883,12 +5858,12 @@
       <c r="AI27" s="13"/>
     </row>
     <row r="28" spans="1:90" s="8" customFormat="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A28" s="155">
+      <c r="A28" s="139">
         <f>COUNTA(C8:C27)</f>
         <v>0</v>
       </c>
-      <c r="B28" s="155"/>
-      <c r="C28" s="155"/>
+      <c r="B28" s="139"/>
+      <c r="C28" s="139"/>
       <c r="D28" s="26"/>
       <c r="E28" s="22">
         <f>SUM(E8:E27)</f>
@@ -6177,30 +6152,30 @@
       <c r="CL30" s="1"/>
     </row>
     <row r="31" spans="1:90" s="48" customFormat="1" ht="17.100000000000001" customHeight="1">
-      <c r="A31" s="156" t="s">
+      <c r="A31" s="140" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="156"/>
-      <c r="C31" s="156"/>
-      <c r="D31" s="156"/>
-      <c r="E31" s="156"/>
-      <c r="F31" s="156"/>
-      <c r="G31" s="156"/>
-      <c r="H31" s="156"/>
-      <c r="I31" s="156"/>
-      <c r="J31" s="156"/>
-      <c r="K31" s="156"/>
-      <c r="L31" s="156"/>
-      <c r="M31" s="156"/>
-      <c r="N31" s="156"/>
-      <c r="O31" s="156"/>
-      <c r="P31" s="156"/>
-      <c r="Q31" s="156"/>
-      <c r="R31" s="156"/>
-      <c r="S31" s="156"/>
-      <c r="T31" s="156"/>
-      <c r="U31" s="156"/>
-      <c r="V31" s="156"/>
+      <c r="B31" s="140"/>
+      <c r="C31" s="140"/>
+      <c r="D31" s="140"/>
+      <c r="E31" s="140"/>
+      <c r="F31" s="140"/>
+      <c r="G31" s="140"/>
+      <c r="H31" s="140"/>
+      <c r="I31" s="140"/>
+      <c r="J31" s="140"/>
+      <c r="K31" s="140"/>
+      <c r="L31" s="140"/>
+      <c r="M31" s="140"/>
+      <c r="N31" s="140"/>
+      <c r="O31" s="140"/>
+      <c r="P31" s="140"/>
+      <c r="Q31" s="140"/>
+      <c r="R31" s="140"/>
+      <c r="S31" s="140"/>
+      <c r="T31" s="140"/>
+      <c r="U31" s="140"/>
+      <c r="V31" s="140"/>
       <c r="W31" s="2"/>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
@@ -6271,30 +6246,30 @@
       <c r="CL31" s="1"/>
     </row>
     <row r="32" spans="1:90" s="48" customFormat="1" ht="17.100000000000001" customHeight="1">
-      <c r="A32" s="157" t="s">
+      <c r="A32" s="141" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="157"/>
-      <c r="C32" s="157"/>
-      <c r="D32" s="157"/>
-      <c r="E32" s="157"/>
-      <c r="F32" s="157"/>
-      <c r="G32" s="157"/>
-      <c r="H32" s="157"/>
-      <c r="I32" s="157"/>
-      <c r="J32" s="157"/>
-      <c r="K32" s="157"/>
-      <c r="L32" s="157"/>
-      <c r="M32" s="157"/>
-      <c r="N32" s="157"/>
-      <c r="O32" s="157"/>
-      <c r="P32" s="157"/>
-      <c r="Q32" s="157"/>
-      <c r="R32" s="157"/>
-      <c r="S32" s="157"/>
-      <c r="T32" s="157"/>
-      <c r="U32" s="157"/>
-      <c r="V32" s="157"/>
+      <c r="B32" s="141"/>
+      <c r="C32" s="141"/>
+      <c r="D32" s="141"/>
+      <c r="E32" s="141"/>
+      <c r="F32" s="141"/>
+      <c r="G32" s="141"/>
+      <c r="H32" s="141"/>
+      <c r="I32" s="141"/>
+      <c r="J32" s="141"/>
+      <c r="K32" s="141"/>
+      <c r="L32" s="141"/>
+      <c r="M32" s="141"/>
+      <c r="N32" s="141"/>
+      <c r="O32" s="141"/>
+      <c r="P32" s="141"/>
+      <c r="Q32" s="141"/>
+      <c r="R32" s="141"/>
+      <c r="S32" s="141"/>
+      <c r="T32" s="141"/>
+      <c r="U32" s="141"/>
+      <c r="V32" s="141"/>
       <c r="W32" s="2"/>
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
@@ -6365,30 +6340,30 @@
       <c r="CL32" s="1"/>
     </row>
     <row r="33" spans="1:90" s="48" customFormat="1" ht="17.100000000000001" customHeight="1">
-      <c r="A33" s="157" t="s">
+      <c r="A33" s="141" t="s">
         <v>4</v>
       </c>
-      <c r="B33" s="157"/>
-      <c r="C33" s="157"/>
-      <c r="D33" s="157"/>
-      <c r="E33" s="157"/>
-      <c r="F33" s="157"/>
-      <c r="G33" s="157"/>
-      <c r="H33" s="157"/>
-      <c r="I33" s="157"/>
-      <c r="J33" s="157"/>
-      <c r="K33" s="157"/>
-      <c r="L33" s="157"/>
-      <c r="M33" s="157"/>
-      <c r="N33" s="157"/>
-      <c r="O33" s="157"/>
-      <c r="P33" s="157"/>
-      <c r="Q33" s="157"/>
-      <c r="R33" s="157"/>
-      <c r="S33" s="157"/>
-      <c r="T33" s="157"/>
-      <c r="U33" s="157"/>
-      <c r="V33" s="157"/>
+      <c r="B33" s="141"/>
+      <c r="C33" s="141"/>
+      <c r="D33" s="141"/>
+      <c r="E33" s="141"/>
+      <c r="F33" s="141"/>
+      <c r="G33" s="141"/>
+      <c r="H33" s="141"/>
+      <c r="I33" s="141"/>
+      <c r="J33" s="141"/>
+      <c r="K33" s="141"/>
+      <c r="L33" s="141"/>
+      <c r="M33" s="141"/>
+      <c r="N33" s="141"/>
+      <c r="O33" s="141"/>
+      <c r="P33" s="141"/>
+      <c r="Q33" s="141"/>
+      <c r="R33" s="141"/>
+      <c r="S33" s="141"/>
+      <c r="T33" s="141"/>
+      <c r="U33" s="141"/>
+      <c r="V33" s="141"/>
       <c r="W33" s="2"/>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
@@ -6459,30 +6434,30 @@
       <c r="CL33" s="1"/>
     </row>
     <row r="34" spans="1:90" s="48" customFormat="1" ht="17.100000000000001" customHeight="1">
-      <c r="A34" s="157" t="s">
+      <c r="A34" s="141" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="157"/>
-      <c r="C34" s="157"/>
-      <c r="D34" s="157"/>
-      <c r="E34" s="157"/>
-      <c r="F34" s="157"/>
-      <c r="G34" s="157"/>
-      <c r="H34" s="157"/>
-      <c r="I34" s="157"/>
-      <c r="J34" s="157"/>
-      <c r="K34" s="157"/>
-      <c r="L34" s="157"/>
-      <c r="M34" s="157"/>
-      <c r="N34" s="157"/>
-      <c r="O34" s="157"/>
-      <c r="P34" s="157"/>
-      <c r="Q34" s="157"/>
-      <c r="R34" s="157"/>
-      <c r="S34" s="157"/>
-      <c r="T34" s="157"/>
-      <c r="U34" s="157"/>
-      <c r="V34" s="157"/>
+      <c r="B34" s="141"/>
+      <c r="C34" s="141"/>
+      <c r="D34" s="141"/>
+      <c r="E34" s="141"/>
+      <c r="F34" s="141"/>
+      <c r="G34" s="141"/>
+      <c r="H34" s="141"/>
+      <c r="I34" s="141"/>
+      <c r="J34" s="141"/>
+      <c r="K34" s="141"/>
+      <c r="L34" s="141"/>
+      <c r="M34" s="141"/>
+      <c r="N34" s="141"/>
+      <c r="O34" s="141"/>
+      <c r="P34" s="141"/>
+      <c r="Q34" s="141"/>
+      <c r="R34" s="141"/>
+      <c r="S34" s="141"/>
+      <c r="T34" s="141"/>
+      <c r="U34" s="141"/>
+      <c r="V34" s="141"/>
       <c r="W34" s="2"/>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
@@ -6651,7 +6626,7 @@
       <c r="B36" s="62"/>
       <c r="C36" s="62"/>
       <c r="D36" s="63"/>
-      <c r="E36" s="153"/>
+      <c r="E36" s="137"/>
       <c r="F36" s="64"/>
       <c r="G36" s="65" t="s">
         <v>3</v>
@@ -6745,7 +6720,7 @@
       <c r="B37" s="62"/>
       <c r="C37" s="62"/>
       <c r="D37" s="63"/>
-      <c r="E37" s="154"/>
+      <c r="E37" s="138"/>
       <c r="F37" s="64"/>
       <c r="G37" s="65" t="s">
         <v>33</v>
@@ -19877,17 +19852,13 @@
   </sheetData>
   <sheetProtection insertRows="0"/>
   <mergeCells count="34">
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A31:V31"/>
-    <mergeCell ref="A32:V32"/>
-    <mergeCell ref="A33:V33"/>
-    <mergeCell ref="A34:V34"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:F2"/>
-    <mergeCell ref="G1:J2"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="L1:R2"/>
+    <mergeCell ref="S6:S7"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="N6:N7"/>
     <mergeCell ref="T4:T7"/>
     <mergeCell ref="U4:U7"/>
     <mergeCell ref="V4:V7"/>
@@ -19904,13 +19875,17 @@
     <mergeCell ref="O6:P6"/>
     <mergeCell ref="Q6:Q7"/>
     <mergeCell ref="R6:R7"/>
-    <mergeCell ref="S6:S7"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:F2"/>
+    <mergeCell ref="G1:J2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="L1:R2"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A31:V31"/>
+    <mergeCell ref="A32:V32"/>
+    <mergeCell ref="A33:V33"/>
+    <mergeCell ref="A34:V34"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="9">

</xml_diff>